<commit_message>
Adding streamlit library for fast web interface
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -446,7 +446,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Remaining</t>
+          <t>Result</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -465,14 +465,14 @@
         <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Needs Checking; Unclear pack (Pwdr/Soln); needs checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -486,14 +486,14 @@
         <v>5</v>
       </c>
       <c r="C3" t="n">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Needs Checking; Unclear pack (Pwdr/Soln); needs checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -507,14 +507,14 @@
         <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -528,14 +528,14 @@
         <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>20</v>
+        <v>220</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -549,14 +549,14 @@
         <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>300</v>
+        <v>475</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -570,14 +570,14 @@
         <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>175</v>
+        <v>475</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -591,14 +591,14 @@
         <v>2</v>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -612,14 +612,14 @@
         <v>5</v>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -633,14 +633,14 @@
         <v>5</v>
       </c>
       <c r="C10" t="n">
-        <v>11</v>
+        <v>422</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -654,14 +654,14 @@
         <v>5</v>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>422</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -675,14 +675,14 @@
         <v>2</v>
       </c>
       <c r="C12" t="n">
-        <v>401</v>
+        <v>422</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Exact Match</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         <v>3</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>422</v>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -717,14 +717,14 @@
         <v>3</v>
       </c>
       <c r="C14" t="n">
-        <v>401</v>
+        <v>422</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -738,14 +738,14 @@
         <v>5</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>422</v>
       </c>
       <c r="D15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -759,14 +759,14 @@
         <v>4</v>
       </c>
       <c r="C16" t="n">
-        <v>277</v>
+        <v>767</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -780,14 +780,14 @@
         <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>200</v>
+        <v>767</v>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -801,14 +801,14 @@
         <v>5</v>
       </c>
       <c r="C18" t="n">
-        <v>5</v>
+        <v>181</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -822,14 +822,14 @@
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>5</v>
+        <v>181</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -843,14 +843,14 @@
         <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>6</v>
+        <v>181</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -864,14 +864,14 @@
         <v>3</v>
       </c>
       <c r="C21" t="n">
-        <v>65</v>
+        <v>181</v>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -913,7 +913,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -927,14 +927,14 @@
         <v>5</v>
       </c>
       <c r="C24" t="n">
-        <v>15</v>
+        <v>580</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -948,14 +948,14 @@
         <v>5</v>
       </c>
       <c r="C25" t="n">
-        <v>15</v>
+        <v>580</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -969,14 +969,14 @@
         <v>5</v>
       </c>
       <c r="C26" t="n">
-        <v>2</v>
+        <v>580</v>
       </c>
       <c r="D26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -990,14 +990,14 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>300</v>
+        <v>580</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1011,14 +1011,14 @@
         <v>5</v>
       </c>
       <c r="C28" t="n">
-        <v>15</v>
+        <v>580</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1032,14 +1032,14 @@
         <v>5</v>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>580</v>
       </c>
       <c r="D29" t="n">
         <v>5</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1053,14 +1053,14 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>255</v>
+        <v>580</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1074,14 +1074,14 @@
         <v>3</v>
       </c>
       <c r="C31" t="n">
-        <v>15</v>
+        <v>580</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1095,14 +1095,14 @@
         <v>3</v>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>580</v>
       </c>
       <c r="D32" t="n">
         <v>3</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1119,11 +1119,11 @@
         <v>150</v>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1133,18 +1133,14 @@
           <t>Atenolol 100 mg Tablet 100's ZENOBLOC-50</t>
         </is>
       </c>
-      <c r="B34" t="n">
-        <v>0</v>
-      </c>
+      <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
-        <v>78</v>
-      </c>
-      <c r="D34" t="n">
-        <v>0</v>
-      </c>
+        <v>278</v>
+      </c>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>No allocation</t>
         </is>
       </c>
     </row>
@@ -1158,14 +1154,14 @@
         <v>2</v>
       </c>
       <c r="C35" t="n">
-        <v>200</v>
+        <v>278</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1179,14 +1175,14 @@
         <v>3</v>
       </c>
       <c r="C36" t="n">
-        <v>300</v>
+        <v>1192</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1200,14 +1196,14 @@
         <v>4</v>
       </c>
       <c r="C37" t="n">
-        <v>340</v>
+        <v>1192</v>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1221,14 +1217,14 @@
         <v>4</v>
       </c>
       <c r="C38" t="n">
-        <v>352</v>
+        <v>1192</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1242,14 +1238,14 @@
         <v>2</v>
       </c>
       <c r="C39" t="n">
-        <v>200</v>
+        <v>1192</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1263,14 +1259,14 @@
         <v>5</v>
       </c>
       <c r="C40" t="n">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1284,14 +1280,14 @@
         <v>5</v>
       </c>
       <c r="C41" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="D41" t="n">
         <v>0</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Exact Match</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1305,14 +1301,14 @@
         <v>2</v>
       </c>
       <c r="C42" t="n">
-        <v>195</v>
+        <v>560</v>
       </c>
       <c r="D42" t="n">
         <v>0</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1326,14 +1322,14 @@
         <v>2</v>
       </c>
       <c r="C43" t="n">
-        <v>195</v>
+        <v>560</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1347,14 +1343,14 @@
         <v>2</v>
       </c>
       <c r="C44" t="n">
-        <v>170</v>
+        <v>560</v>
       </c>
       <c r="D44" t="n">
         <v>0</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1371,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1388,9 +1384,7 @@
       <c r="B46" t="n">
         <v>2</v>
       </c>
-      <c r="C46" t="n">
-        <v>0</v>
-      </c>
+      <c r="C46" t="inlineStr"/>
       <c r="D46" t="n">
         <v>2</v>
       </c>
@@ -1417,7 +1411,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1434,11 +1428,11 @@
         <v>2</v>
       </c>
       <c r="D48" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1452,14 +1446,14 @@
         <v>5</v>
       </c>
       <c r="C49" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D49" t="n">
         <v>5</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1473,14 +1467,14 @@
         <v>5</v>
       </c>
       <c r="C50" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1494,14 +1488,14 @@
         <v>3</v>
       </c>
       <c r="C51" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="D51" t="n">
         <v>0</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1515,14 +1509,14 @@
         <v>2</v>
       </c>
       <c r="C52" t="n">
-        <v>300</v>
+        <v>440</v>
       </c>
       <c r="D52" t="n">
         <v>0</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1536,14 +1530,14 @@
         <v>3</v>
       </c>
       <c r="C53" t="n">
-        <v>300</v>
+        <v>440</v>
       </c>
       <c r="D53" t="n">
         <v>0</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1557,14 +1551,14 @@
         <v>3</v>
       </c>
       <c r="C54" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
       <c r="D54" t="n">
         <v>0</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1578,14 +1572,14 @@
         <v>3</v>
       </c>
       <c r="C55" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
       <c r="D55" t="n">
         <v>0</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1600,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1627,7 +1621,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1637,18 +1631,14 @@
           <t>CARBOCISTEINE Drops</t>
         </is>
       </c>
-      <c r="B58" t="n">
-        <v>0</v>
-      </c>
+      <c r="B58" t="inlineStr"/>
       <c r="C58" t="n">
-        <v>0</v>
-      </c>
-      <c r="D58" t="n">
-        <v>0</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>No allocation</t>
         </is>
       </c>
     </row>
@@ -1662,14 +1652,14 @@
         <v>5</v>
       </c>
       <c r="C59" t="n">
-        <v>0</v>
+        <v>176</v>
       </c>
       <c r="D59" t="n">
         <v>5</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1683,14 +1673,14 @@
         <v>5</v>
       </c>
       <c r="C60" t="n">
-        <v>3</v>
+        <v>176</v>
       </c>
       <c r="D60" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1704,14 +1694,14 @@
         <v>5</v>
       </c>
       <c r="C61" t="n">
-        <v>3</v>
+        <v>176</v>
       </c>
       <c r="D61" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1725,14 +1715,14 @@
         <v>3</v>
       </c>
       <c r="C62" t="n">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="D62" t="n">
         <v>1</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1753,7 +1743,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1763,18 +1753,14 @@
           <t>Carvedilol 12.5mg</t>
         </is>
       </c>
-      <c r="B64" t="n">
-        <v>0</v>
-      </c>
+      <c r="B64" t="inlineStr"/>
       <c r="C64" t="n">
-        <v>0</v>
-      </c>
-      <c r="D64" t="n">
-        <v>0</v>
-      </c>
+        <v>407</v>
+      </c>
+      <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>No allocation</t>
         </is>
       </c>
     </row>
@@ -1788,14 +1774,14 @@
         <v>4</v>
       </c>
       <c r="C65" t="n">
-        <v>0</v>
+        <v>407</v>
       </c>
       <c r="D65" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1809,14 +1795,14 @@
         <v>5</v>
       </c>
       <c r="C66" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D66" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1830,14 +1816,14 @@
         <v>5</v>
       </c>
       <c r="C67" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1851,14 +1837,14 @@
         <v>5</v>
       </c>
       <c r="C68" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1872,14 +1858,14 @@
         <v>5</v>
       </c>
       <c r="C69" t="n">
-        <v>6</v>
+        <v>407</v>
       </c>
       <c r="D69" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1893,14 +1879,14 @@
         <v>5</v>
       </c>
       <c r="C70" t="n">
-        <v>5</v>
+        <v>407</v>
       </c>
       <c r="D70" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1914,14 +1900,14 @@
         <v>2</v>
       </c>
       <c r="C71" t="n">
-        <v>196</v>
+        <v>407</v>
       </c>
       <c r="D71" t="n">
         <v>0</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1935,14 +1921,14 @@
         <v>5</v>
       </c>
       <c r="C72" t="n">
-        <v>5</v>
+        <v>407</v>
       </c>
       <c r="D72" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -1956,14 +1942,14 @@
         <v>2</v>
       </c>
       <c r="C73" t="n">
-        <v>195</v>
+        <v>407</v>
       </c>
       <c r="D73" t="n">
         <v>0</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -1973,18 +1959,14 @@
           <t>Cefixime 400mg Tab</t>
         </is>
       </c>
-      <c r="B74" t="n">
-        <v>0</v>
-      </c>
+      <c r="B74" t="inlineStr"/>
       <c r="C74" t="n">
-        <v>0</v>
-      </c>
-      <c r="D74" t="n">
-        <v>0</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>No allocation</t>
         </is>
       </c>
     </row>
@@ -2005,7 +1987,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Audit pack: complex count; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2019,14 +2001,14 @@
         <v>5</v>
       </c>
       <c r="C76" t="n">
-        <v>5</v>
+        <v>51</v>
       </c>
       <c r="D76" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2040,14 +2022,14 @@
         <v>5</v>
       </c>
       <c r="C77" t="n">
-        <v>4</v>
+        <v>51</v>
       </c>
       <c r="D77" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2061,14 +2043,14 @@
         <v>5</v>
       </c>
       <c r="C78" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="D78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2082,14 +2064,14 @@
         <v>4</v>
       </c>
       <c r="C79" t="n">
-        <v>331</v>
+        <v>628</v>
       </c>
       <c r="D79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2103,14 +2085,14 @@
         <v>3</v>
       </c>
       <c r="C80" t="n">
-        <v>297</v>
+        <v>628</v>
       </c>
       <c r="D80" t="n">
         <v>0</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2124,14 +2106,14 @@
         <v>5</v>
       </c>
       <c r="C81" t="n">
-        <v>497</v>
+        <v>944</v>
       </c>
       <c r="D81" t="n">
         <v>0</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2145,14 +2127,14 @@
         <v>5</v>
       </c>
       <c r="C82" t="n">
-        <v>0</v>
+        <v>944</v>
       </c>
       <c r="D82" t="n">
         <v>5</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2166,14 +2148,14 @@
         <v>5</v>
       </c>
       <c r="C83" t="n">
-        <v>7</v>
+        <v>944</v>
       </c>
       <c r="D83" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2190,11 +2172,11 @@
         <v>4</v>
       </c>
       <c r="D84" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2208,14 +2190,14 @@
         <v>3</v>
       </c>
       <c r="C85" t="n">
-        <v>539</v>
+        <v>1528</v>
       </c>
       <c r="D85" t="n">
         <v>0</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2229,14 +2211,14 @@
         <v>3</v>
       </c>
       <c r="C86" t="n">
-        <v>539</v>
+        <v>1528</v>
       </c>
       <c r="D86" t="n">
         <v>0</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2239,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2270,9 +2252,7 @@
       <c r="B88" t="n">
         <v>5</v>
       </c>
-      <c r="C88" t="n">
-        <v>0</v>
-      </c>
+      <c r="C88" t="inlineStr"/>
       <c r="D88" t="n">
         <v>5</v>
       </c>
@@ -2299,7 +2279,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2300,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2321,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2355,14 +2335,14 @@
         <v>5</v>
       </c>
       <c r="C92" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D92" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2376,14 +2356,14 @@
         <v>5</v>
       </c>
       <c r="C93" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D93" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2384,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2421,11 +2401,11 @@
         <v>3</v>
       </c>
       <c r="D95" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2435,18 +2415,14 @@
           <t>Clonidine 150mg Tab 100's</t>
         </is>
       </c>
-      <c r="B96" t="n">
-        <v>0</v>
-      </c>
+      <c r="B96" t="inlineStr"/>
       <c r="C96" t="n">
-        <v>0</v>
-      </c>
-      <c r="D96" t="n">
-        <v>0</v>
-      </c>
+        <v>296</v>
+      </c>
+      <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>No allocation</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2443,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2484,11 +2460,11 @@
         <v>5</v>
       </c>
       <c r="D98" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2502,14 +2478,14 @@
         <v>5</v>
       </c>
       <c r="C99" t="n">
-        <v>5</v>
+        <v>210</v>
       </c>
       <c r="D99" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2523,14 +2499,14 @@
         <v>5</v>
       </c>
       <c r="C100" t="n">
-        <v>5</v>
+        <v>210</v>
       </c>
       <c r="D100" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2544,14 +2520,14 @@
         <v>2</v>
       </c>
       <c r="C101" t="n">
-        <v>0</v>
+        <v>210</v>
       </c>
       <c r="D101" t="n">
         <v>2</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2565,14 +2541,14 @@
         <v>5</v>
       </c>
       <c r="C102" t="n">
-        <v>0</v>
+        <v>2943</v>
       </c>
       <c r="D102" t="n">
         <v>5</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2586,14 +2562,14 @@
         <v>5</v>
       </c>
       <c r="C103" t="n">
-        <v>0</v>
+        <v>2943</v>
       </c>
       <c r="D103" t="n">
         <v>5</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2607,14 +2583,14 @@
         <v>5</v>
       </c>
       <c r="C104" t="n">
-        <v>5</v>
+        <v>2943</v>
       </c>
       <c r="D104" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2628,14 +2604,14 @@
         <v>4</v>
       </c>
       <c r="C105" t="n">
-        <v>34</v>
+        <v>2943</v>
       </c>
       <c r="D105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2656,7 +2632,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2670,14 +2646,14 @@
         <v>5</v>
       </c>
       <c r="C107" t="n">
-        <v>5</v>
+        <v>192</v>
       </c>
       <c r="D107" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2691,14 +2667,14 @@
         <v>5</v>
       </c>
       <c r="C108" t="n">
-        <v>5</v>
+        <v>192</v>
       </c>
       <c r="D108" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2712,14 +2688,14 @@
         <v>2</v>
       </c>
       <c r="C109" t="n">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="D109" t="n">
         <v>0</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2740,7 +2716,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2754,14 +2730,14 @@
         <v>2</v>
       </c>
       <c r="C111" t="n">
-        <v>130</v>
+        <v>310</v>
       </c>
       <c r="D111" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2775,14 +2751,14 @@
         <v>2</v>
       </c>
       <c r="C112" t="n">
-        <v>180</v>
+        <v>310</v>
       </c>
       <c r="D112" t="n">
         <v>0</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2799,11 +2775,11 @@
         <v>5</v>
       </c>
       <c r="D113" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2800,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2838,14 +2814,14 @@
         <v>5</v>
       </c>
       <c r="C115" t="n">
-        <v>0</v>
+        <v>205</v>
       </c>
       <c r="D115" t="n">
         <v>5</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2859,14 +2835,14 @@
         <v>2</v>
       </c>
       <c r="C116" t="n">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="D116" t="n">
         <v>0</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2880,14 +2856,14 @@
         <v>5</v>
       </c>
       <c r="C117" t="n">
-        <v>5</v>
+        <v>253</v>
       </c>
       <c r="D117" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -2901,14 +2877,14 @@
         <v>2</v>
       </c>
       <c r="C118" t="n">
-        <v>188</v>
+        <v>253</v>
       </c>
       <c r="D118" t="n">
         <v>0</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2905,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2943,14 +2919,14 @@
         <v>2</v>
       </c>
       <c r="C120" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="D120" t="n">
         <v>0</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2964,14 +2940,14 @@
         <v>2</v>
       </c>
       <c r="C121" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="D121" t="n">
         <v>0</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -2988,11 +2964,11 @@
         <v>7</v>
       </c>
       <c r="D122" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3006,14 +2982,14 @@
         <v>5</v>
       </c>
       <c r="C123" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D123" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -3027,14 +3003,14 @@
         <v>5</v>
       </c>
       <c r="C124" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="D124" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -3048,14 +3024,14 @@
         <v>2</v>
       </c>
       <c r="C125" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="D125" t="n">
         <v>2</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3052,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3090,14 +3066,14 @@
         <v>2</v>
       </c>
       <c r="C127" t="n">
-        <v>110</v>
+        <v>200</v>
       </c>
       <c r="D127" t="n">
         <v>0</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Exact Match</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3111,14 +3087,14 @@
         <v>3</v>
       </c>
       <c r="C128" t="n">
-        <v>90</v>
+        <v>200</v>
       </c>
       <c r="D128" t="n">
         <v>0</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3128,18 +3104,14 @@
           <t>Etoricoxib 60mg</t>
         </is>
       </c>
-      <c r="B129" t="n">
-        <v>0</v>
-      </c>
+      <c r="B129" t="inlineStr"/>
       <c r="C129" t="n">
-        <v>0</v>
-      </c>
-      <c r="D129" t="n">
-        <v>0</v>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="D129" t="inlineStr"/>
       <c r="E129" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>No allocation</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3132,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3174,14 +3146,14 @@
         <v>3</v>
       </c>
       <c r="C131" t="n">
-        <v>13</v>
+        <v>103</v>
       </c>
       <c r="D131" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3195,14 +3167,14 @@
         <v>3</v>
       </c>
       <c r="C132" t="n">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="D132" t="n">
         <v>0</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3215,9 +3187,7 @@
       <c r="B133" t="n">
         <v>2</v>
       </c>
-      <c r="C133" t="n">
-        <v>0</v>
-      </c>
+      <c r="C133" t="inlineStr"/>
       <c r="D133" t="n">
         <v>2</v>
       </c>
@@ -3233,18 +3203,14 @@
           <t>Fenofibrate 160mg</t>
         </is>
       </c>
-      <c r="B134" t="n">
-        <v>0</v>
-      </c>
+      <c r="B134" t="inlineStr"/>
       <c r="C134" t="n">
-        <v>0</v>
-      </c>
-      <c r="D134" t="n">
-        <v>0</v>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="D134" t="inlineStr"/>
       <c r="E134" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>No allocation</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3231,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3279,14 +3245,14 @@
         <v>5</v>
       </c>
       <c r="C136" t="n">
-        <v>0</v>
+        <v>410</v>
       </c>
       <c r="D136" t="n">
         <v>5</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -3300,14 +3266,14 @@
         <v>2</v>
       </c>
       <c r="C137" t="n">
-        <v>0</v>
+        <v>410</v>
       </c>
       <c r="D137" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3321,14 +3287,14 @@
         <v>2</v>
       </c>
       <c r="C138" t="n">
-        <v>90</v>
+        <v>410</v>
       </c>
       <c r="D138" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Check pack size; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3342,14 +3308,14 @@
         <v>2</v>
       </c>
       <c r="C139" t="n">
-        <v>165</v>
+        <v>410</v>
       </c>
       <c r="D139" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -3363,14 +3329,14 @@
         <v>2</v>
       </c>
       <c r="C140" t="n">
-        <v>145</v>
+        <v>410</v>
       </c>
       <c r="D140" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3384,14 +3350,14 @@
         <v>5</v>
       </c>
       <c r="C141" t="n">
-        <v>5</v>
+        <v>410</v>
       </c>
       <c r="D141" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -3404,9 +3370,7 @@
       <c r="B142" t="n">
         <v>3</v>
       </c>
-      <c r="C142" t="n">
-        <v>0</v>
-      </c>
+      <c r="C142" t="inlineStr"/>
       <c r="D142" t="n">
         <v>3</v>
       </c>
@@ -3433,7 +3397,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3454,7 +3418,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Audit pack: complex count; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3468,14 +3432,14 @@
         <v>3</v>
       </c>
       <c r="C145" t="n">
-        <v>170</v>
+        <v>260</v>
       </c>
       <c r="D145" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3489,14 +3453,14 @@
         <v>2</v>
       </c>
       <c r="C146" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="D146" t="n">
         <v>0</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3510,14 +3474,14 @@
         <v>3</v>
       </c>
       <c r="C147" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="D147" t="n">
         <v>0</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3538,7 +3502,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3555,11 +3519,11 @@
         <v>1</v>
       </c>
       <c r="D149" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Needs Checking; Unclear pack (Pwdr/Soln); needs checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3544,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3594,14 +3558,14 @@
         <v>2</v>
       </c>
       <c r="C151" t="n">
-        <v>122</v>
+        <v>275</v>
       </c>
       <c r="D151" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3615,14 +3579,14 @@
         <v>2</v>
       </c>
       <c r="C152" t="n">
-        <v>153</v>
+        <v>275</v>
       </c>
       <c r="D152" t="n">
         <v>0</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3636,14 +3600,14 @@
         <v>2</v>
       </c>
       <c r="C153" t="n">
-        <v>200</v>
+        <v>590</v>
       </c>
       <c r="D153" t="n">
         <v>0</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3657,14 +3621,14 @@
         <v>2</v>
       </c>
       <c r="C154" t="n">
-        <v>200</v>
+        <v>590</v>
       </c>
       <c r="D154" t="n">
         <v>0</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3678,14 +3642,14 @@
         <v>5</v>
       </c>
       <c r="C155" t="n">
-        <v>0</v>
+        <v>410</v>
       </c>
       <c r="D155" t="n">
         <v>5</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -3699,14 +3663,14 @@
         <v>5</v>
       </c>
       <c r="C156" t="n">
-        <v>0</v>
+        <v>410</v>
       </c>
       <c r="D156" t="n">
         <v>5</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -3723,11 +3687,11 @@
         <v>5</v>
       </c>
       <c r="D157" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3712,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3758,15 +3722,9 @@
           <t>HNBB Syrup60ml</t>
         </is>
       </c>
-      <c r="B159" t="n">
-        <v>0</v>
-      </c>
-      <c r="C159" t="n">
-        <v>0</v>
-      </c>
-      <c r="D159" t="n">
-        <v>0</v>
-      </c>
+      <c r="B159" t="inlineStr"/>
+      <c r="C159" t="inlineStr"/>
+      <c r="D159" t="inlineStr"/>
       <c r="E159" t="inlineStr">
         <is>
           <t>No match found</t>
@@ -3783,14 +3741,14 @@
         <v>5</v>
       </c>
       <c r="C160" t="n">
-        <v>3</v>
+        <v>352</v>
       </c>
       <c r="D160" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -3804,14 +3762,14 @@
         <v>2</v>
       </c>
       <c r="C161" t="n">
-        <v>161</v>
+        <v>352</v>
       </c>
       <c r="D161" t="n">
         <v>0</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3821,18 +3779,14 @@
           <t>Irbesartan 300mg 100's</t>
         </is>
       </c>
-      <c r="B162" t="n">
-        <v>0</v>
-      </c>
+      <c r="B162" t="inlineStr"/>
       <c r="C162" t="n">
-        <v>100</v>
-      </c>
-      <c r="D162" t="n">
-        <v>0</v>
-      </c>
+        <v>254</v>
+      </c>
+      <c r="D162" t="inlineStr"/>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>No allocation</t>
         </is>
       </c>
     </row>
@@ -3846,14 +3800,14 @@
         <v>2</v>
       </c>
       <c r="C163" t="n">
-        <v>154</v>
+        <v>254</v>
       </c>
       <c r="D163" t="n">
         <v>0</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3866,9 +3820,7 @@
       <c r="B164" t="n">
         <v>2</v>
       </c>
-      <c r="C164" t="n">
-        <v>0</v>
-      </c>
+      <c r="C164" t="inlineStr"/>
       <c r="D164" t="n">
         <v>2</v>
       </c>
@@ -3888,14 +3840,14 @@
         <v>2</v>
       </c>
       <c r="C165" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D165" t="n">
         <v>2</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3909,14 +3861,14 @@
         <v>5</v>
       </c>
       <c r="C166" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D166" t="n">
         <v>5</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -3930,14 +3882,14 @@
         <v>5</v>
       </c>
       <c r="C167" t="n">
-        <v>11</v>
+        <v>343</v>
       </c>
       <c r="D167" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -3951,14 +3903,14 @@
         <v>2</v>
       </c>
       <c r="C168" t="n">
-        <v>160</v>
+        <v>343</v>
       </c>
       <c r="D168" t="n">
         <v>0</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -3972,14 +3924,14 @@
         <v>5</v>
       </c>
       <c r="C169" t="n">
-        <v>11</v>
+        <v>343</v>
       </c>
       <c r="D169" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -3993,14 +3945,14 @@
         <v>2</v>
       </c>
       <c r="C170" t="n">
-        <v>172</v>
+        <v>343</v>
       </c>
       <c r="D170" t="n">
         <v>0</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4021,7 +3973,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4042,7 +3994,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4063,7 +4015,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4077,14 +4029,14 @@
         <v>2</v>
       </c>
       <c r="C174" t="n">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="D174" t="n">
         <v>0</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4098,14 +4050,14 @@
         <v>5</v>
       </c>
       <c r="C175" t="n">
-        <v>5</v>
+        <v>195</v>
       </c>
       <c r="D175" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -4119,14 +4071,14 @@
         <v>2</v>
       </c>
       <c r="C176" t="n">
-        <v>200</v>
+        <v>1019</v>
       </c>
       <c r="D176" t="n">
         <v>0</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4140,14 +4092,14 @@
         <v>3</v>
       </c>
       <c r="C177" t="n">
-        <v>213</v>
+        <v>1019</v>
       </c>
       <c r="D177" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4161,14 +4113,14 @@
         <v>4</v>
       </c>
       <c r="C178" t="n">
-        <v>106</v>
+        <v>1019</v>
       </c>
       <c r="D178" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4182,14 +4134,14 @@
         <v>3</v>
       </c>
       <c r="C179" t="n">
-        <v>200</v>
+        <v>1019</v>
       </c>
       <c r="D179" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4203,14 +4155,14 @@
         <v>2</v>
       </c>
       <c r="C180" t="n">
-        <v>200</v>
+        <v>1019</v>
       </c>
       <c r="D180" t="n">
         <v>0</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4224,14 +4176,14 @@
         <v>5</v>
       </c>
       <c r="C181" t="n">
-        <v>5</v>
+        <v>205</v>
       </c>
       <c r="D181" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -4244,9 +4196,7 @@
       <c r="B182" t="n">
         <v>2</v>
       </c>
-      <c r="C182" t="n">
-        <v>0</v>
-      </c>
+      <c r="C182" t="inlineStr"/>
       <c r="D182" t="n">
         <v>2</v>
       </c>
@@ -4266,14 +4216,14 @@
         <v>3</v>
       </c>
       <c r="C183" t="n">
-        <v>300</v>
+        <v>453</v>
       </c>
       <c r="D183" t="n">
         <v>0</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4287,14 +4237,14 @@
         <v>4</v>
       </c>
       <c r="C184" t="n">
-        <v>149</v>
+        <v>453</v>
       </c>
       <c r="D184" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4308,14 +4258,14 @@
         <v>5</v>
       </c>
       <c r="C185" t="n">
-        <v>4</v>
+        <v>453</v>
       </c>
       <c r="D185" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -4336,7 +4286,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4350,14 +4300,14 @@
         <v>5</v>
       </c>
       <c r="C187" t="n">
-        <v>5</v>
+        <v>205</v>
       </c>
       <c r="D187" t="n">
         <v>0</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4371,14 +4321,14 @@
         <v>3</v>
       </c>
       <c r="C188" t="n">
-        <v>300</v>
+        <v>745</v>
       </c>
       <c r="D188" t="n">
         <v>0</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4392,14 +4342,14 @@
         <v>5</v>
       </c>
       <c r="C189" t="n">
-        <v>445</v>
+        <v>745</v>
       </c>
       <c r="D189" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4413,14 +4363,14 @@
         <v>5</v>
       </c>
       <c r="C190" t="n">
-        <v>4</v>
+        <v>204</v>
       </c>
       <c r="D190" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -4434,14 +4384,14 @@
         <v>2</v>
       </c>
       <c r="C191" t="n">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="D191" t="n">
         <v>0</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4455,14 +4405,14 @@
         <v>5</v>
       </c>
       <c r="C192" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D192" t="n">
         <v>5</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -4479,11 +4429,11 @@
         <v>5</v>
       </c>
       <c r="D193" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -4497,14 +4447,14 @@
         <v>3</v>
       </c>
       <c r="C194" t="n">
-        <v>150</v>
+        <v>696</v>
       </c>
       <c r="D194" t="n">
         <v>0</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4518,14 +4468,14 @@
         <v>4</v>
       </c>
       <c r="C195" t="n">
-        <v>56</v>
+        <v>696</v>
       </c>
       <c r="D195" t="n">
         <v>0</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Audit pack: complex count; Check pack size; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4539,14 +4489,14 @@
         <v>2</v>
       </c>
       <c r="C196" t="n">
-        <v>200</v>
+        <v>696</v>
       </c>
       <c r="D196" t="n">
         <v>0</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4560,14 +4510,14 @@
         <v>5</v>
       </c>
       <c r="C197" t="n">
-        <v>0</v>
+        <v>759</v>
       </c>
       <c r="D197" t="n">
         <v>5</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -4581,14 +4531,14 @@
         <v>5</v>
       </c>
       <c r="C198" t="n">
-        <v>10</v>
+        <v>754</v>
       </c>
       <c r="D198" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -4602,14 +4552,14 @@
         <v>2</v>
       </c>
       <c r="C199" t="n">
-        <v>534</v>
+        <v>749</v>
       </c>
       <c r="D199" t="n">
         <v>0</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4623,14 +4573,14 @@
         <v>3</v>
       </c>
       <c r="C200" t="n">
-        <v>534</v>
+        <v>749</v>
       </c>
       <c r="D200" t="n">
         <v>0</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4644,14 +4594,14 @@
         <v>3</v>
       </c>
       <c r="C201" t="n">
-        <v>534</v>
+        <v>749</v>
       </c>
       <c r="D201" t="n">
         <v>0</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4665,14 +4615,14 @@
         <v>2</v>
       </c>
       <c r="C202" t="n">
-        <v>200</v>
+        <v>749</v>
       </c>
       <c r="D202" t="n">
         <v>0</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4686,14 +4636,14 @@
         <v>5</v>
       </c>
       <c r="C203" t="n">
-        <v>10</v>
+        <v>749</v>
       </c>
       <c r="D203" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -4707,14 +4657,14 @@
         <v>5</v>
       </c>
       <c r="C204" t="n">
-        <v>10</v>
+        <v>749</v>
       </c>
       <c r="D204" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -4731,11 +4681,11 @@
         <v>5</v>
       </c>
       <c r="D205" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -4748,9 +4698,7 @@
       <c r="B206" t="n">
         <v>3</v>
       </c>
-      <c r="C206" t="n">
-        <v>0</v>
-      </c>
+      <c r="C206" t="inlineStr"/>
       <c r="D206" t="n">
         <v>3</v>
       </c>
@@ -4769,9 +4717,7 @@
       <c r="B207" t="n">
         <v>3</v>
       </c>
-      <c r="C207" t="n">
-        <v>0</v>
-      </c>
+      <c r="C207" t="inlineStr"/>
       <c r="D207" t="n">
         <v>3</v>
       </c>
@@ -4791,14 +4737,14 @@
         <v>2</v>
       </c>
       <c r="C208" t="n">
-        <v>0</v>
+        <v>384</v>
       </c>
       <c r="D208" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4812,14 +4758,14 @@
         <v>3</v>
       </c>
       <c r="C209" t="n">
-        <v>0</v>
+        <v>283</v>
       </c>
       <c r="D209" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4840,7 +4786,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4861,7 +4807,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4875,14 +4821,14 @@
         <v>2</v>
       </c>
       <c r="C212" t="n">
-        <v>183</v>
+        <v>387</v>
       </c>
       <c r="D212" t="n">
         <v>0</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4896,14 +4842,14 @@
         <v>2</v>
       </c>
       <c r="C213" t="n">
-        <v>204</v>
+        <v>387</v>
       </c>
       <c r="D213" t="n">
         <v>0</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4917,14 +4863,14 @@
         <v>3</v>
       </c>
       <c r="C214" t="n">
-        <v>56</v>
+        <v>97</v>
       </c>
       <c r="D214" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4938,14 +4884,14 @@
         <v>2</v>
       </c>
       <c r="C215" t="n">
-        <v>60</v>
+        <v>156</v>
       </c>
       <c r="D215" t="n">
         <v>0</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4959,14 +4905,14 @@
         <v>2</v>
       </c>
       <c r="C216" t="n">
-        <v>96</v>
+        <v>156</v>
       </c>
       <c r="D216" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -4980,14 +4926,14 @@
         <v>2</v>
       </c>
       <c r="C217" t="n">
-        <v>194</v>
+        <v>1528</v>
       </c>
       <c r="D217" t="n">
         <v>0</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5001,14 +4947,14 @@
         <v>2</v>
       </c>
       <c r="C218" t="n">
-        <v>353</v>
+        <v>786</v>
       </c>
       <c r="D218" t="n">
         <v>0</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5022,14 +4968,14 @@
         <v>5</v>
       </c>
       <c r="C219" t="n">
-        <v>0</v>
+        <v>786</v>
       </c>
       <c r="D219" t="n">
         <v>5</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -5043,14 +4989,14 @@
         <v>2</v>
       </c>
       <c r="C220" t="n">
-        <v>353</v>
+        <v>786</v>
       </c>
       <c r="D220" t="n">
         <v>0</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5064,14 +5010,14 @@
         <v>5</v>
       </c>
       <c r="C221" t="n">
-        <v>2</v>
+        <v>786</v>
       </c>
       <c r="D221" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -5085,14 +5031,14 @@
         <v>5</v>
       </c>
       <c r="C222" t="n">
-        <v>1</v>
+        <v>786</v>
       </c>
       <c r="D222" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5106,14 +5052,14 @@
         <v>5</v>
       </c>
       <c r="C223" t="n">
-        <v>1</v>
+        <v>786</v>
       </c>
       <c r="D223" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5127,14 +5073,14 @@
         <v>5</v>
       </c>
       <c r="C224" t="n">
-        <v>2</v>
+        <v>786</v>
       </c>
       <c r="D224" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -5148,14 +5094,14 @@
         <v>5</v>
       </c>
       <c r="C225" t="n">
-        <v>428</v>
+        <v>786</v>
       </c>
       <c r="D225" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5169,14 +5115,14 @@
         <v>5</v>
       </c>
       <c r="C226" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D226" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -5190,14 +5136,14 @@
         <v>5</v>
       </c>
       <c r="C227" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D227" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -5214,11 +5160,11 @@
         <v>4</v>
       </c>
       <c r="D228" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -5232,14 +5178,14 @@
         <v>2</v>
       </c>
       <c r="C229" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="D229" t="n">
         <v>1</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5253,14 +5199,14 @@
         <v>2</v>
       </c>
       <c r="C230" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="D230" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5274,14 +5220,14 @@
         <v>5</v>
       </c>
       <c r="C231" t="n">
-        <v>5</v>
+        <v>541</v>
       </c>
       <c r="D231" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -5295,14 +5241,14 @@
         <v>2</v>
       </c>
       <c r="C232" t="n">
-        <v>148</v>
+        <v>541</v>
       </c>
       <c r="D232" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5316,14 +5262,14 @@
         <v>2</v>
       </c>
       <c r="C233" t="n">
-        <v>196</v>
+        <v>541</v>
       </c>
       <c r="D233" t="n">
         <v>0</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5337,14 +5283,14 @@
         <v>2</v>
       </c>
       <c r="C234" t="n">
-        <v>192</v>
+        <v>541</v>
       </c>
       <c r="D234" t="n">
         <v>0</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5311,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5379,14 +5325,14 @@
         <v>2</v>
       </c>
       <c r="C236" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="D236" t="n">
         <v>0</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5400,14 +5346,14 @@
         <v>2</v>
       </c>
       <c r="C237" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="D237" t="n">
         <v>0</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5374,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5442,14 +5388,14 @@
         <v>2</v>
       </c>
       <c r="C239" t="n">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="D239" t="n">
         <v>0</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5463,14 +5409,14 @@
         <v>2</v>
       </c>
       <c r="C240" t="n">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="D240" t="n">
         <v>0</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5484,14 +5430,14 @@
         <v>2</v>
       </c>
       <c r="C241" t="n">
-        <v>200</v>
+        <v>530</v>
       </c>
       <c r="D241" t="n">
         <v>0</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5505,14 +5451,14 @@
         <v>2</v>
       </c>
       <c r="C242" t="n">
-        <v>130</v>
+        <v>530</v>
       </c>
       <c r="D242" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5526,14 +5472,14 @@
         <v>2</v>
       </c>
       <c r="C243" t="n">
-        <v>200</v>
+        <v>1131</v>
       </c>
       <c r="D243" t="n">
         <v>0</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5547,14 +5493,14 @@
         <v>2</v>
       </c>
       <c r="C244" t="n">
-        <v>0</v>
+        <v>1131</v>
       </c>
       <c r="D244" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5568,14 +5514,14 @@
         <v>3</v>
       </c>
       <c r="C245" t="n">
-        <v>3</v>
+        <v>931</v>
       </c>
       <c r="D245" t="n">
         <v>0</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5589,14 +5535,14 @@
         <v>2</v>
       </c>
       <c r="C246" t="n">
-        <v>642</v>
+        <v>931</v>
       </c>
       <c r="D246" t="n">
         <v>0</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>Capsule vs Tablet; review; Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5610,14 +5556,14 @@
         <v>2</v>
       </c>
       <c r="C247" t="n">
-        <v>0</v>
+        <v>931</v>
       </c>
       <c r="D247" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5631,14 +5577,14 @@
         <v>5</v>
       </c>
       <c r="C248" t="n">
-        <v>442</v>
+        <v>931</v>
       </c>
       <c r="D248" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5652,14 +5598,14 @@
         <v>2</v>
       </c>
       <c r="C249" t="n">
-        <v>200</v>
+        <v>931</v>
       </c>
       <c r="D249" t="n">
         <v>0</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5673,14 +5619,14 @@
         <v>3</v>
       </c>
       <c r="C250" t="n">
-        <v>0</v>
+        <v>931</v>
       </c>
       <c r="D250" t="n">
         <v>3</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -5694,14 +5640,14 @@
         <v>3</v>
       </c>
       <c r="C251" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D251" t="n">
         <v>3</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -5722,7 +5668,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5736,14 +5682,14 @@
         <v>5</v>
       </c>
       <c r="C253" t="n">
-        <v>50</v>
+        <v>78</v>
       </c>
       <c r="D253" t="n">
         <v>0</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5757,14 +5703,14 @@
         <v>2</v>
       </c>
       <c r="C254" t="n">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="D254" t="n">
         <v>0</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5781,11 +5727,11 @@
         <v>5</v>
       </c>
       <c r="D255" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -5799,14 +5745,14 @@
         <v>2</v>
       </c>
       <c r="C256" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="D256" t="n">
         <v>0</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5820,14 +5766,14 @@
         <v>3</v>
       </c>
       <c r="C257" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="D257" t="n">
         <v>0</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5841,14 +5787,14 @@
         <v>5</v>
       </c>
       <c r="C258" t="n">
-        <v>0</v>
+        <v>387</v>
       </c>
       <c r="D258" t="n">
         <v>5</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -5865,11 +5811,11 @@
         <v>150</v>
       </c>
       <c r="D259" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5890,7 +5836,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5904,14 +5850,14 @@
         <v>5</v>
       </c>
       <c r="C261" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D261" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -5925,14 +5871,14 @@
         <v>2</v>
       </c>
       <c r="C262" t="n">
-        <v>200</v>
+        <v>365</v>
       </c>
       <c r="D262" t="n">
         <v>0</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5953,7 +5899,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5974,7 +5920,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Exact Match</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -5988,14 +5934,14 @@
         <v>2</v>
       </c>
       <c r="C265" t="n">
-        <v>170</v>
+        <v>1648</v>
       </c>
       <c r="D265" t="n">
         <v>0</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -6009,14 +5955,14 @@
         <v>2</v>
       </c>
       <c r="C266" t="n">
-        <v>824</v>
+        <v>1648</v>
       </c>
       <c r="D266" t="n">
         <v>0</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Capsule vs Tablet; review; Check pack size; Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -6030,14 +5976,14 @@
         <v>3</v>
       </c>
       <c r="C267" t="n">
-        <v>300</v>
+        <v>1079</v>
       </c>
       <c r="D267" t="n">
         <v>0</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -6051,14 +5997,14 @@
         <v>5</v>
       </c>
       <c r="C268" t="n">
-        <v>5</v>
+        <v>839</v>
       </c>
       <c r="D268" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Needs Checking</t>
+          <t>Needs checking (pack size unknown)</t>
         </is>
       </c>
     </row>
@@ -6072,14 +6018,14 @@
         <v>3</v>
       </c>
       <c r="C269" t="n">
-        <v>624</v>
+        <v>839</v>
       </c>
       <c r="D269" t="n">
         <v>0</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Check pack size; Combined multiple brands; Needs Checking</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>
@@ -6093,14 +6039,14 @@
         <v>2</v>
       </c>
       <c r="C270" t="n">
-        <v>0</v>
+        <v>839</v>
       </c>
       <c r="D270" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>No match found</t>
+          <t>Exact match</t>
         </is>
       </c>
     </row>

</xml_diff>